<commit_message>
Refactor benchmark parameters to require explicit dataset folder and run count
</commit_message>
<xml_diff>
--- a/results/benchmark_results.xlsx
+++ b/results/benchmark_results.xlsx
@@ -471,10 +471,10 @@
         <v>1</v>
       </c>
       <c r="D2" t="n">
-        <v>7961</v>
+        <v>8306</v>
       </c>
       <c r="E2" t="n">
-        <v>0.2838186999999834</v>
+        <v>0.2958247999999912</v>
       </c>
     </row>
     <row r="3">
@@ -492,10 +492,10 @@
         <v>1</v>
       </c>
       <c r="D3" t="n">
-        <v>8710</v>
+        <v>9171</v>
       </c>
       <c r="E3" t="n">
-        <v>7.372638100000131</v>
+        <v>4.565246500000285</v>
       </c>
     </row>
     <row r="4">
@@ -516,7 +516,7 @@
         <v>7679</v>
       </c>
       <c r="E4" t="n">
-        <v>14.74633160000008</v>
+        <v>8.004324700000325</v>
       </c>
     </row>
     <row r="5">
@@ -534,10 +534,10 @@
         <v>1</v>
       </c>
       <c r="D5" t="n">
-        <v>689</v>
+        <v>693</v>
       </c>
       <c r="E5" t="n">
-        <v>7.824557799999866</v>
+        <v>3.463330300000052</v>
       </c>
     </row>
     <row r="6">
@@ -555,10 +555,10 @@
         <v>1</v>
       </c>
       <c r="D6" t="n">
-        <v>941</v>
+        <v>918</v>
       </c>
       <c r="E6" t="n">
-        <v>26.68744790000005</v>
+        <v>11.22962730000017</v>
       </c>
     </row>
     <row r="7">
@@ -576,10 +576,10 @@
         <v>1</v>
       </c>
       <c r="D7" t="n">
-        <v>694</v>
+        <v>679</v>
       </c>
       <c r="E7" t="n">
-        <v>89.09790040000007</v>
+        <v>56.03252470000007</v>
       </c>
     </row>
     <row r="8">
@@ -597,10 +597,10 @@
         <v>1</v>
       </c>
       <c r="D8" t="n">
-        <v>23569</v>
+        <v>22355</v>
       </c>
       <c r="E8" t="n">
-        <v>4.444546299999729</v>
+        <v>5.33241709999993</v>
       </c>
     </row>
     <row r="9">
@@ -618,10 +618,10 @@
         <v>1</v>
       </c>
       <c r="D9" t="n">
-        <v>33330</v>
+        <v>32338</v>
       </c>
       <c r="E9" t="n">
-        <v>11.19634570000017</v>
+        <v>12.04212490000009</v>
       </c>
     </row>
     <row r="10">
@@ -639,10 +639,10 @@
         <v>1</v>
       </c>
       <c r="D10" t="n">
-        <v>23173</v>
+        <v>22560</v>
       </c>
       <c r="E10" t="n">
-        <v>51.88828330000024</v>
+        <v>118.0442397000002</v>
       </c>
     </row>
     <row r="11">
@@ -660,10 +660,10 @@
         <v>1</v>
       </c>
       <c r="D11" t="n">
-        <v>1380</v>
+        <v>1364</v>
       </c>
       <c r="E11" t="n">
-        <v>3.30304120000028</v>
+        <v>9.9755339000003</v>
       </c>
     </row>
     <row r="12">
@@ -681,10 +681,10 @@
         <v>1</v>
       </c>
       <c r="D12" t="n">
-        <v>1856</v>
+        <v>2044</v>
       </c>
       <c r="E12" t="n">
-        <v>10.52190449999989</v>
+        <v>25.6808845999999</v>
       </c>
     </row>
     <row r="13">
@@ -702,10 +702,10 @@
         <v>1</v>
       </c>
       <c r="D13" t="n">
-        <v>1272</v>
+        <v>1292</v>
       </c>
       <c r="E13" t="n">
-        <v>48.98392400000012</v>
+        <v>119.7659322</v>
       </c>
     </row>
     <row r="14">
@@ -723,10 +723,10 @@
         <v>1</v>
       </c>
       <c r="D14" t="n">
-        <v>734</v>
+        <v>737</v>
       </c>
       <c r="E14" t="n">
-        <v>0.7974186999999802</v>
+        <v>2.213883899999928</v>
       </c>
     </row>
     <row r="15">
@@ -744,10 +744,10 @@
         <v>1</v>
       </c>
       <c r="D15" t="n">
-        <v>897</v>
+        <v>920</v>
       </c>
       <c r="E15" t="n">
-        <v>6.221123499999976</v>
+        <v>15.47965359999989</v>
       </c>
     </row>
     <row r="16">
@@ -765,10 +765,10 @@
         <v>1</v>
       </c>
       <c r="D16" t="n">
-        <v>716</v>
+        <v>714</v>
       </c>
       <c r="E16" t="n">
-        <v>17.89616269999988</v>
+        <v>48.94194920000018</v>
       </c>
     </row>
   </sheetData>
@@ -834,17 +834,17 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>7961</v>
+        <v>8306</v>
       </c>
       <c r="D2" t="n">
-        <v>7961</v>
+        <v>8306</v>
       </c>
       <c r="E2" t="n">
-        <v>7961</v>
+        <v>8306</v>
       </c>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="n">
-        <v>0.2838186999999834</v>
+        <v>0.2958247999999912</v>
       </c>
     </row>
     <row r="3">
@@ -869,7 +869,7 @@
       </c>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="n">
-        <v>14.74633160000008</v>
+        <v>8.004324700000325</v>
       </c>
     </row>
     <row r="4">
@@ -884,17 +884,17 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>8710</v>
+        <v>9171</v>
       </c>
       <c r="D4" t="n">
-        <v>8710</v>
+        <v>9171</v>
       </c>
       <c r="E4" t="n">
-        <v>8710</v>
+        <v>9171</v>
       </c>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="n">
-        <v>7.372638100000131</v>
+        <v>4.565246500000285</v>
       </c>
     </row>
     <row r="5">
@@ -909,17 +909,17 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>689</v>
+        <v>693</v>
       </c>
       <c r="D5" t="n">
-        <v>689</v>
+        <v>693</v>
       </c>
       <c r="E5" t="n">
-        <v>689</v>
+        <v>693</v>
       </c>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="n">
-        <v>7.824557799999866</v>
+        <v>3.463330300000052</v>
       </c>
     </row>
     <row r="6">
@@ -934,17 +934,17 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>694</v>
+        <v>679</v>
       </c>
       <c r="D6" t="n">
-        <v>694</v>
+        <v>679</v>
       </c>
       <c r="E6" t="n">
-        <v>694</v>
+        <v>679</v>
       </c>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="n">
-        <v>89.09790040000007</v>
+        <v>56.03252470000007</v>
       </c>
     </row>
     <row r="7">
@@ -959,17 +959,17 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>941</v>
+        <v>918</v>
       </c>
       <c r="D7" t="n">
-        <v>941</v>
+        <v>918</v>
       </c>
       <c r="E7" t="n">
-        <v>941</v>
+        <v>918</v>
       </c>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="n">
-        <v>26.68744790000005</v>
+        <v>11.22962730000017</v>
       </c>
     </row>
     <row r="8">
@@ -984,17 +984,17 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>23569</v>
+        <v>22355</v>
       </c>
       <c r="D8" t="n">
-        <v>23569</v>
+        <v>22355</v>
       </c>
       <c r="E8" t="n">
-        <v>23569</v>
+        <v>22355</v>
       </c>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="n">
-        <v>4.444546299999729</v>
+        <v>5.33241709999993</v>
       </c>
     </row>
     <row r="9">
@@ -1009,17 +1009,17 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>23173</v>
+        <v>22560</v>
       </c>
       <c r="D9" t="n">
-        <v>23173</v>
+        <v>22560</v>
       </c>
       <c r="E9" t="n">
-        <v>23173</v>
+        <v>22560</v>
       </c>
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="n">
-        <v>51.88828330000024</v>
+        <v>118.0442397000002</v>
       </c>
     </row>
     <row r="10">
@@ -1034,17 +1034,17 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>33330</v>
+        <v>32338</v>
       </c>
       <c r="D10" t="n">
-        <v>33330</v>
+        <v>32338</v>
       </c>
       <c r="E10" t="n">
-        <v>33330</v>
+        <v>32338</v>
       </c>
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="n">
-        <v>11.19634570000017</v>
+        <v>12.04212490000009</v>
       </c>
     </row>
     <row r="11">
@@ -1059,17 +1059,17 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>1380</v>
+        <v>1364</v>
       </c>
       <c r="D11" t="n">
-        <v>1380</v>
+        <v>1364</v>
       </c>
       <c r="E11" t="n">
-        <v>1380</v>
+        <v>1364</v>
       </c>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="n">
-        <v>3.30304120000028</v>
+        <v>9.9755339000003</v>
       </c>
     </row>
     <row r="12">
@@ -1084,17 +1084,17 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>1272</v>
+        <v>1292</v>
       </c>
       <c r="D12" t="n">
-        <v>1272</v>
+        <v>1292</v>
       </c>
       <c r="E12" t="n">
-        <v>1272</v>
+        <v>1292</v>
       </c>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="n">
-        <v>48.98392400000012</v>
+        <v>119.7659322</v>
       </c>
     </row>
     <row r="13">
@@ -1109,17 +1109,17 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>1856</v>
+        <v>2044</v>
       </c>
       <c r="D13" t="n">
-        <v>1856</v>
+        <v>2044</v>
       </c>
       <c r="E13" t="n">
-        <v>1856</v>
+        <v>2044</v>
       </c>
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="n">
-        <v>10.52190449999989</v>
+        <v>25.6808845999999</v>
       </c>
     </row>
     <row r="14">
@@ -1134,17 +1134,17 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>734</v>
+        <v>737</v>
       </c>
       <c r="D14" t="n">
-        <v>734</v>
+        <v>737</v>
       </c>
       <c r="E14" t="n">
-        <v>734</v>
+        <v>737</v>
       </c>
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="n">
-        <v>0.7974186999999802</v>
+        <v>2.213883899999928</v>
       </c>
     </row>
     <row r="15">
@@ -1159,17 +1159,17 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>716</v>
+        <v>714</v>
       </c>
       <c r="D15" t="n">
-        <v>716</v>
+        <v>714</v>
       </c>
       <c r="E15" t="n">
-        <v>716</v>
+        <v>714</v>
       </c>
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="n">
-        <v>17.89616269999988</v>
+        <v>48.94194920000018</v>
       </c>
     </row>
     <row r="16">
@@ -1184,17 +1184,17 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>897</v>
+        <v>920</v>
       </c>
       <c r="D16" t="n">
-        <v>897</v>
+        <v>920</v>
       </c>
       <c r="E16" t="n">
-        <v>897</v>
+        <v>920</v>
       </c>
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="n">
-        <v>6.221123499999976</v>
+        <v>15.47965359999989</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix transition probabilities calculation in Ant Colony algorithm and remove unused random seed in main.py
</commit_message>
<xml_diff>
--- a/results/benchmark_results.xlsx
+++ b/results/benchmark_results.xlsx
@@ -471,10 +471,10 @@
         <v>1</v>
       </c>
       <c r="D2" t="n">
-        <v>8306</v>
+        <v>8051</v>
       </c>
       <c r="E2" t="n">
-        <v>0.2958247999999912</v>
+        <v>0.3019074000003457</v>
       </c>
     </row>
     <row r="3">
@@ -492,10 +492,10 @@
         <v>1</v>
       </c>
       <c r="D3" t="n">
-        <v>9171</v>
+        <v>9146</v>
       </c>
       <c r="E3" t="n">
-        <v>4.565246500000285</v>
+        <v>4.893026499999905</v>
       </c>
     </row>
     <row r="4">
@@ -513,10 +513,10 @@
         <v>1</v>
       </c>
       <c r="D4" t="n">
-        <v>7679</v>
+        <v>7674</v>
       </c>
       <c r="E4" t="n">
-        <v>8.004324700000325</v>
+        <v>11.46315210000012</v>
       </c>
     </row>
     <row r="5">
@@ -534,10 +534,10 @@
         <v>1</v>
       </c>
       <c r="D5" t="n">
-        <v>693</v>
+        <v>672</v>
       </c>
       <c r="E5" t="n">
-        <v>3.463330300000052</v>
+        <v>7.471019100000376</v>
       </c>
     </row>
     <row r="6">
@@ -555,10 +555,10 @@
         <v>1</v>
       </c>
       <c r="D6" t="n">
-        <v>918</v>
+        <v>938</v>
       </c>
       <c r="E6" t="n">
-        <v>11.22962730000017</v>
+        <v>14.46527900000001</v>
       </c>
     </row>
     <row r="7">
@@ -576,10 +576,10 @@
         <v>1</v>
       </c>
       <c r="D7" t="n">
-        <v>679</v>
+        <v>687</v>
       </c>
       <c r="E7" t="n">
-        <v>56.03252470000007</v>
+        <v>125.0588582999999</v>
       </c>
     </row>
     <row r="8">
@@ -597,10 +597,10 @@
         <v>1</v>
       </c>
       <c r="D8" t="n">
-        <v>22355</v>
+        <v>22646</v>
       </c>
       <c r="E8" t="n">
-        <v>5.33241709999993</v>
+        <v>8.813124799999969</v>
       </c>
     </row>
     <row r="9">
@@ -618,10 +618,10 @@
         <v>1</v>
       </c>
       <c r="D9" t="n">
-        <v>32338</v>
+        <v>40945</v>
       </c>
       <c r="E9" t="n">
-        <v>12.04212490000009</v>
+        <v>25.47362050000083</v>
       </c>
     </row>
     <row r="10">
@@ -639,10 +639,10 @@
         <v>1</v>
       </c>
       <c r="D10" t="n">
-        <v>22560</v>
+        <v>23108</v>
       </c>
       <c r="E10" t="n">
-        <v>118.0442397000002</v>
+        <v>99.46364229999926</v>
       </c>
     </row>
     <row r="11">
@@ -660,10 +660,10 @@
         <v>1</v>
       </c>
       <c r="D11" t="n">
-        <v>1364</v>
+        <v>1338</v>
       </c>
       <c r="E11" t="n">
-        <v>9.9755339000003</v>
+        <v>4.128855799999656</v>
       </c>
     </row>
     <row r="12">
@@ -681,10 +681,10 @@
         <v>1</v>
       </c>
       <c r="D12" t="n">
-        <v>2044</v>
+        <v>2128</v>
       </c>
       <c r="E12" t="n">
-        <v>25.6808845999999</v>
+        <v>16.57324160000007</v>
       </c>
     </row>
     <row r="13">
@@ -702,10 +702,10 @@
         <v>1</v>
       </c>
       <c r="D13" t="n">
-        <v>1292</v>
+        <v>1286</v>
       </c>
       <c r="E13" t="n">
-        <v>119.7659322</v>
+        <v>90.52328229999966</v>
       </c>
     </row>
     <row r="14">
@@ -723,10 +723,10 @@
         <v>1</v>
       </c>
       <c r="D14" t="n">
-        <v>737</v>
+        <v>742</v>
       </c>
       <c r="E14" t="n">
-        <v>2.213883899999928</v>
+        <v>0.9917675000006057</v>
       </c>
     </row>
     <row r="15">
@@ -744,10 +744,10 @@
         <v>1</v>
       </c>
       <c r="D15" t="n">
-        <v>920</v>
+        <v>915</v>
       </c>
       <c r="E15" t="n">
-        <v>15.47965359999989</v>
+        <v>6.9923974000003</v>
       </c>
     </row>
     <row r="16">
@@ -765,10 +765,10 @@
         <v>1</v>
       </c>
       <c r="D16" t="n">
-        <v>714</v>
+        <v>713</v>
       </c>
       <c r="E16" t="n">
-        <v>48.94194920000018</v>
+        <v>20.49216140000044</v>
       </c>
     </row>
   </sheetData>
@@ -834,17 +834,17 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>8306</v>
+        <v>8051</v>
       </c>
       <c r="D2" t="n">
-        <v>8306</v>
+        <v>8051</v>
       </c>
       <c r="E2" t="n">
-        <v>8306</v>
+        <v>8051</v>
       </c>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="n">
-        <v>0.2958247999999912</v>
+        <v>0.3019074000003457</v>
       </c>
     </row>
     <row r="3">
@@ -859,17 +859,17 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>7679</v>
+        <v>7674</v>
       </c>
       <c r="D3" t="n">
-        <v>7679</v>
+        <v>7674</v>
       </c>
       <c r="E3" t="n">
-        <v>7679</v>
+        <v>7674</v>
       </c>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="n">
-        <v>8.004324700000325</v>
+        <v>11.46315210000012</v>
       </c>
     </row>
     <row r="4">
@@ -884,17 +884,17 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>9171</v>
+        <v>9146</v>
       </c>
       <c r="D4" t="n">
-        <v>9171</v>
+        <v>9146</v>
       </c>
       <c r="E4" t="n">
-        <v>9171</v>
+        <v>9146</v>
       </c>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="n">
-        <v>4.565246500000285</v>
+        <v>4.893026499999905</v>
       </c>
     </row>
     <row r="5">
@@ -909,17 +909,17 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>693</v>
+        <v>672</v>
       </c>
       <c r="D5" t="n">
-        <v>693</v>
+        <v>672</v>
       </c>
       <c r="E5" t="n">
-        <v>693</v>
+        <v>672</v>
       </c>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="n">
-        <v>3.463330300000052</v>
+        <v>7.471019100000376</v>
       </c>
     </row>
     <row r="6">
@@ -934,17 +934,17 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>679</v>
+        <v>687</v>
       </c>
       <c r="D6" t="n">
-        <v>679</v>
+        <v>687</v>
       </c>
       <c r="E6" t="n">
-        <v>679</v>
+        <v>687</v>
       </c>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="n">
-        <v>56.03252470000007</v>
+        <v>125.0588582999999</v>
       </c>
     </row>
     <row r="7">
@@ -959,17 +959,17 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>918</v>
+        <v>938</v>
       </c>
       <c r="D7" t="n">
-        <v>918</v>
+        <v>938</v>
       </c>
       <c r="E7" t="n">
-        <v>918</v>
+        <v>938</v>
       </c>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="n">
-        <v>11.22962730000017</v>
+        <v>14.46527900000001</v>
       </c>
     </row>
     <row r="8">
@@ -984,17 +984,17 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>22355</v>
+        <v>22646</v>
       </c>
       <c r="D8" t="n">
-        <v>22355</v>
+        <v>22646</v>
       </c>
       <c r="E8" t="n">
-        <v>22355</v>
+        <v>22646</v>
       </c>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="n">
-        <v>5.33241709999993</v>
+        <v>8.813124799999969</v>
       </c>
     </row>
     <row r="9">
@@ -1009,17 +1009,17 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>22560</v>
+        <v>23108</v>
       </c>
       <c r="D9" t="n">
-        <v>22560</v>
+        <v>23108</v>
       </c>
       <c r="E9" t="n">
-        <v>22560</v>
+        <v>23108</v>
       </c>
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="n">
-        <v>118.0442397000002</v>
+        <v>99.46364229999926</v>
       </c>
     </row>
     <row r="10">
@@ -1034,17 +1034,17 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>32338</v>
+        <v>40945</v>
       </c>
       <c r="D10" t="n">
-        <v>32338</v>
+        <v>40945</v>
       </c>
       <c r="E10" t="n">
-        <v>32338</v>
+        <v>40945</v>
       </c>
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="n">
-        <v>12.04212490000009</v>
+        <v>25.47362050000083</v>
       </c>
     </row>
     <row r="11">
@@ -1059,17 +1059,17 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>1364</v>
+        <v>1338</v>
       </c>
       <c r="D11" t="n">
-        <v>1364</v>
+        <v>1338</v>
       </c>
       <c r="E11" t="n">
-        <v>1364</v>
+        <v>1338</v>
       </c>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="n">
-        <v>9.9755339000003</v>
+        <v>4.128855799999656</v>
       </c>
     </row>
     <row r="12">
@@ -1084,17 +1084,17 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>1292</v>
+        <v>1286</v>
       </c>
       <c r="D12" t="n">
-        <v>1292</v>
+        <v>1286</v>
       </c>
       <c r="E12" t="n">
-        <v>1292</v>
+        <v>1286</v>
       </c>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="n">
-        <v>119.7659322</v>
+        <v>90.52328229999966</v>
       </c>
     </row>
     <row r="13">
@@ -1109,17 +1109,17 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>2044</v>
+        <v>2128</v>
       </c>
       <c r="D13" t="n">
-        <v>2044</v>
+        <v>2128</v>
       </c>
       <c r="E13" t="n">
-        <v>2044</v>
+        <v>2128</v>
       </c>
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="n">
-        <v>25.6808845999999</v>
+        <v>16.57324160000007</v>
       </c>
     </row>
     <row r="14">
@@ -1134,17 +1134,17 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>737</v>
+        <v>742</v>
       </c>
       <c r="D14" t="n">
-        <v>737</v>
+        <v>742</v>
       </c>
       <c r="E14" t="n">
-        <v>737</v>
+        <v>742</v>
       </c>
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="n">
-        <v>2.213883899999928</v>
+        <v>0.9917675000006057</v>
       </c>
     </row>
     <row r="15">
@@ -1159,17 +1159,17 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>714</v>
+        <v>713</v>
       </c>
       <c r="D15" t="n">
-        <v>714</v>
+        <v>713</v>
       </c>
       <c r="E15" t="n">
-        <v>714</v>
+        <v>713</v>
       </c>
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="n">
-        <v>48.94194920000018</v>
+        <v>20.49216140000044</v>
       </c>
     </row>
     <row r="16">
@@ -1184,17 +1184,17 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>920</v>
+        <v>915</v>
       </c>
       <c r="D16" t="n">
-        <v>920</v>
+        <v>915</v>
       </c>
       <c r="E16" t="n">
-        <v>920</v>
+        <v>915</v>
       </c>
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="n">
-        <v>15.47965359999989</v>
+        <v>6.9923974000003</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix visibility matrix calculation to handle zero distances and improve transition probabilities normalization
</commit_message>
<xml_diff>
--- a/results/benchmark_results.xlsx
+++ b/results/benchmark_results.xlsx
@@ -471,10 +471,10 @@
         <v>1</v>
       </c>
       <c r="D2" t="n">
-        <v>8051</v>
+        <v>7955</v>
       </c>
       <c r="E2" t="n">
-        <v>0.3019074000003457</v>
+        <v>0.3334324000006745</v>
       </c>
     </row>
     <row r="3">
@@ -492,10 +492,10 @@
         <v>1</v>
       </c>
       <c r="D3" t="n">
-        <v>9146</v>
+        <v>8495</v>
       </c>
       <c r="E3" t="n">
-        <v>4.893026499999905</v>
+        <v>4.900403800000277</v>
       </c>
     </row>
     <row r="4">
@@ -513,10 +513,10 @@
         <v>1</v>
       </c>
       <c r="D4" t="n">
-        <v>7674</v>
+        <v>7662</v>
       </c>
       <c r="E4" t="n">
-        <v>11.46315210000012</v>
+        <v>12.48907169999984</v>
       </c>
     </row>
     <row r="5">
@@ -534,10 +534,10 @@
         <v>1</v>
       </c>
       <c r="D5" t="n">
-        <v>672</v>
+        <v>675</v>
       </c>
       <c r="E5" t="n">
-        <v>7.471019100000376</v>
+        <v>3.794308999999885</v>
       </c>
     </row>
     <row r="6">
@@ -555,10 +555,10 @@
         <v>1</v>
       </c>
       <c r="D6" t="n">
-        <v>938</v>
+        <v>958</v>
       </c>
       <c r="E6" t="n">
-        <v>14.46527900000001</v>
+        <v>15.42478030000075</v>
       </c>
     </row>
     <row r="7">
@@ -576,10 +576,10 @@
         <v>1</v>
       </c>
       <c r="D7" t="n">
-        <v>687</v>
+        <v>681</v>
       </c>
       <c r="E7" t="n">
-        <v>125.0588582999999</v>
+        <v>129.007764</v>
       </c>
     </row>
     <row r="8">
@@ -597,10 +597,10 @@
         <v>1</v>
       </c>
       <c r="D8" t="n">
-        <v>22646</v>
+        <v>22483</v>
       </c>
       <c r="E8" t="n">
-        <v>8.813124799999969</v>
+        <v>10.74744179999925</v>
       </c>
     </row>
     <row r="9">
@@ -618,10 +618,10 @@
         <v>1</v>
       </c>
       <c r="D9" t="n">
-        <v>40945</v>
+        <v>33203</v>
       </c>
       <c r="E9" t="n">
-        <v>25.47362050000083</v>
+        <v>26.97715880000032</v>
       </c>
     </row>
     <row r="10">
@@ -639,10 +639,10 @@
         <v>1</v>
       </c>
       <c r="D10" t="n">
-        <v>23108</v>
+        <v>22857</v>
       </c>
       <c r="E10" t="n">
-        <v>99.46364229999926</v>
+        <v>131.9376242999997</v>
       </c>
     </row>
     <row r="11">
@@ -660,10 +660,10 @@
         <v>1</v>
       </c>
       <c r="D11" t="n">
-        <v>1338</v>
+        <v>1369</v>
       </c>
       <c r="E11" t="n">
-        <v>4.128855799999656</v>
+        <v>8.247546900000088</v>
       </c>
     </row>
     <row r="12">
@@ -681,10 +681,10 @@
         <v>1</v>
       </c>
       <c r="D12" t="n">
-        <v>2128</v>
+        <v>1888</v>
       </c>
       <c r="E12" t="n">
-        <v>16.57324160000007</v>
+        <v>18.93730810000034</v>
       </c>
     </row>
     <row r="13">
@@ -702,10 +702,10 @@
         <v>1</v>
       </c>
       <c r="D13" t="n">
-        <v>1286</v>
+        <v>1280</v>
       </c>
       <c r="E13" t="n">
-        <v>90.52328229999966</v>
+        <v>119.1917635</v>
       </c>
     </row>
     <row r="14">
@@ -723,10 +723,10 @@
         <v>1</v>
       </c>
       <c r="D14" t="n">
-        <v>742</v>
+        <v>711</v>
       </c>
       <c r="E14" t="n">
-        <v>0.9917675000006057</v>
+        <v>1.885228199999801</v>
       </c>
     </row>
     <row r="15">
@@ -744,10 +744,10 @@
         <v>1</v>
       </c>
       <c r="D15" t="n">
-        <v>915</v>
+        <v>980</v>
       </c>
       <c r="E15" t="n">
-        <v>6.9923974000003</v>
+        <v>15.25094390000049</v>
       </c>
     </row>
     <row r="16">
@@ -765,10 +765,10 @@
         <v>1</v>
       </c>
       <c r="D16" t="n">
-        <v>713</v>
+        <v>719</v>
       </c>
       <c r="E16" t="n">
-        <v>20.49216140000044</v>
+        <v>40.94512949999989</v>
       </c>
     </row>
   </sheetData>
@@ -834,17 +834,17 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>8051</v>
+        <v>7955</v>
       </c>
       <c r="D2" t="n">
-        <v>8051</v>
+        <v>7955</v>
       </c>
       <c r="E2" t="n">
-        <v>8051</v>
+        <v>7955</v>
       </c>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="n">
-        <v>0.3019074000003457</v>
+        <v>0.3334324000006745</v>
       </c>
     </row>
     <row r="3">
@@ -859,17 +859,17 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>7674</v>
+        <v>7662</v>
       </c>
       <c r="D3" t="n">
-        <v>7674</v>
+        <v>7662</v>
       </c>
       <c r="E3" t="n">
-        <v>7674</v>
+        <v>7662</v>
       </c>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="n">
-        <v>11.46315210000012</v>
+        <v>12.48907169999984</v>
       </c>
     </row>
     <row r="4">
@@ -884,17 +884,17 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>9146</v>
+        <v>8495</v>
       </c>
       <c r="D4" t="n">
-        <v>9146</v>
+        <v>8495</v>
       </c>
       <c r="E4" t="n">
-        <v>9146</v>
+        <v>8495</v>
       </c>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="n">
-        <v>4.893026499999905</v>
+        <v>4.900403800000277</v>
       </c>
     </row>
     <row r="5">
@@ -909,17 +909,17 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>672</v>
+        <v>675</v>
       </c>
       <c r="D5" t="n">
-        <v>672</v>
+        <v>675</v>
       </c>
       <c r="E5" t="n">
-        <v>672</v>
+        <v>675</v>
       </c>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="n">
-        <v>7.471019100000376</v>
+        <v>3.794308999999885</v>
       </c>
     </row>
     <row r="6">
@@ -934,17 +934,17 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>687</v>
+        <v>681</v>
       </c>
       <c r="D6" t="n">
-        <v>687</v>
+        <v>681</v>
       </c>
       <c r="E6" t="n">
-        <v>687</v>
+        <v>681</v>
       </c>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="n">
-        <v>125.0588582999999</v>
+        <v>129.007764</v>
       </c>
     </row>
     <row r="7">
@@ -959,17 +959,17 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>938</v>
+        <v>958</v>
       </c>
       <c r="D7" t="n">
-        <v>938</v>
+        <v>958</v>
       </c>
       <c r="E7" t="n">
-        <v>938</v>
+        <v>958</v>
       </c>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="n">
-        <v>14.46527900000001</v>
+        <v>15.42478030000075</v>
       </c>
     </row>
     <row r="8">
@@ -984,17 +984,17 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>22646</v>
+        <v>22483</v>
       </c>
       <c r="D8" t="n">
-        <v>22646</v>
+        <v>22483</v>
       </c>
       <c r="E8" t="n">
-        <v>22646</v>
+        <v>22483</v>
       </c>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="n">
-        <v>8.813124799999969</v>
+        <v>10.74744179999925</v>
       </c>
     </row>
     <row r="9">
@@ -1009,17 +1009,17 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>23108</v>
+        <v>22857</v>
       </c>
       <c r="D9" t="n">
-        <v>23108</v>
+        <v>22857</v>
       </c>
       <c r="E9" t="n">
-        <v>23108</v>
+        <v>22857</v>
       </c>
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="n">
-        <v>99.46364229999926</v>
+        <v>131.9376242999997</v>
       </c>
     </row>
     <row r="10">
@@ -1034,17 +1034,17 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>40945</v>
+        <v>33203</v>
       </c>
       <c r="D10" t="n">
-        <v>40945</v>
+        <v>33203</v>
       </c>
       <c r="E10" t="n">
-        <v>40945</v>
+        <v>33203</v>
       </c>
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="n">
-        <v>25.47362050000083</v>
+        <v>26.97715880000032</v>
       </c>
     </row>
     <row r="11">
@@ -1059,17 +1059,17 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>1338</v>
+        <v>1369</v>
       </c>
       <c r="D11" t="n">
-        <v>1338</v>
+        <v>1369</v>
       </c>
       <c r="E11" t="n">
-        <v>1338</v>
+        <v>1369</v>
       </c>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="n">
-        <v>4.128855799999656</v>
+        <v>8.247546900000088</v>
       </c>
     </row>
     <row r="12">
@@ -1084,17 +1084,17 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>1286</v>
+        <v>1280</v>
       </c>
       <c r="D12" t="n">
-        <v>1286</v>
+        <v>1280</v>
       </c>
       <c r="E12" t="n">
-        <v>1286</v>
+        <v>1280</v>
       </c>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="n">
-        <v>90.52328229999966</v>
+        <v>119.1917635</v>
       </c>
     </row>
     <row r="13">
@@ -1109,17 +1109,17 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>2128</v>
+        <v>1888</v>
       </c>
       <c r="D13" t="n">
-        <v>2128</v>
+        <v>1888</v>
       </c>
       <c r="E13" t="n">
-        <v>2128</v>
+        <v>1888</v>
       </c>
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="n">
-        <v>16.57324160000007</v>
+        <v>18.93730810000034</v>
       </c>
     </row>
     <row r="14">
@@ -1134,17 +1134,17 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>742</v>
+        <v>711</v>
       </c>
       <c r="D14" t="n">
-        <v>742</v>
+        <v>711</v>
       </c>
       <c r="E14" t="n">
-        <v>742</v>
+        <v>711</v>
       </c>
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="n">
-        <v>0.9917675000006057</v>
+        <v>1.885228199999801</v>
       </c>
     </row>
     <row r="15">
@@ -1159,17 +1159,17 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>713</v>
+        <v>719</v>
       </c>
       <c r="D15" t="n">
-        <v>713</v>
+        <v>719</v>
       </c>
       <c r="E15" t="n">
-        <v>713</v>
+        <v>719</v>
       </c>
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="n">
-        <v>20.49216140000044</v>
+        <v>40.94512949999989</v>
       </c>
     </row>
     <row r="16">
@@ -1184,17 +1184,17 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>915</v>
+        <v>980</v>
       </c>
       <c r="D16" t="n">
-        <v>915</v>
+        <v>980</v>
       </c>
       <c r="E16" t="n">
-        <v>915</v>
+        <v>980</v>
       </c>
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="n">
-        <v>6.9923974000003</v>
+        <v>15.25094390000049</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update benchmark results and binary for improved performance
</commit_message>
<xml_diff>
--- a/results/benchmark_results.xlsx
+++ b/results/benchmark_results.xlsx
@@ -471,10 +471,10 @@
         <v>1</v>
       </c>
       <c r="D2" t="n">
-        <v>7955</v>
+        <v>7871</v>
       </c>
       <c r="E2" t="n">
-        <v>0.3334324000006745</v>
+        <v>0.2966114000009838</v>
       </c>
     </row>
     <row r="3">
@@ -492,10 +492,10 @@
         <v>1</v>
       </c>
       <c r="D3" t="n">
-        <v>8495</v>
+        <v>8342</v>
       </c>
       <c r="E3" t="n">
-        <v>4.900403800000277</v>
+        <v>5.168920899999648</v>
       </c>
     </row>
     <row r="4">
@@ -513,10 +513,10 @@
         <v>1</v>
       </c>
       <c r="D4" t="n">
-        <v>7662</v>
+        <v>7674</v>
       </c>
       <c r="E4" t="n">
-        <v>12.48907169999984</v>
+        <v>8.998690500000521</v>
       </c>
     </row>
     <row r="5">
@@ -534,10 +534,10 @@
         <v>1</v>
       </c>
       <c r="D5" t="n">
-        <v>675</v>
+        <v>686</v>
       </c>
       <c r="E5" t="n">
-        <v>3.794308999999885</v>
+        <v>4.112357500000144</v>
       </c>
     </row>
     <row r="6">
@@ -555,10 +555,10 @@
         <v>1</v>
       </c>
       <c r="D6" t="n">
-        <v>958</v>
+        <v>1009</v>
       </c>
       <c r="E6" t="n">
-        <v>15.42478030000075</v>
+        <v>12.76222730000154</v>
       </c>
     </row>
     <row r="7">
@@ -576,10 +576,10 @@
         <v>1</v>
       </c>
       <c r="D7" t="n">
-        <v>681</v>
+        <v>689</v>
       </c>
       <c r="E7" t="n">
-        <v>129.007764</v>
+        <v>65.01397750000069</v>
       </c>
     </row>
     <row r="8">
@@ -597,10 +597,10 @@
         <v>1</v>
       </c>
       <c r="D8" t="n">
-        <v>22483</v>
+        <v>22442</v>
       </c>
       <c r="E8" t="n">
-        <v>10.74744179999925</v>
+        <v>4.652482800000143</v>
       </c>
     </row>
     <row r="9">
@@ -618,10 +618,10 @@
         <v>1</v>
       </c>
       <c r="D9" t="n">
-        <v>33203</v>
+        <v>33940</v>
       </c>
       <c r="E9" t="n">
-        <v>26.97715880000032</v>
+        <v>12.71414080000068</v>
       </c>
     </row>
     <row r="10">
@@ -639,10 +639,10 @@
         <v>1</v>
       </c>
       <c r="D10" t="n">
-        <v>22857</v>
+        <v>22879</v>
       </c>
       <c r="E10" t="n">
-        <v>131.9376242999997</v>
+        <v>62.5200748999996</v>
       </c>
     </row>
     <row r="11">
@@ -660,10 +660,10 @@
         <v>1</v>
       </c>
       <c r="D11" t="n">
-        <v>1369</v>
+        <v>1314</v>
       </c>
       <c r="E11" t="n">
-        <v>8.247546900000088</v>
+        <v>4.023495299999922</v>
       </c>
     </row>
     <row r="12">
@@ -681,10 +681,10 @@
         <v>1</v>
       </c>
       <c r="D12" t="n">
-        <v>1888</v>
+        <v>1853</v>
       </c>
       <c r="E12" t="n">
-        <v>18.93730810000034</v>
+        <v>12.24914619999981</v>
       </c>
     </row>
     <row r="13">
@@ -702,10 +702,10 @@
         <v>1</v>
       </c>
       <c r="D13" t="n">
-        <v>1280</v>
+        <v>1292</v>
       </c>
       <c r="E13" t="n">
-        <v>119.1917635</v>
+        <v>56.92731110000022</v>
       </c>
     </row>
     <row r="14">
@@ -723,10 +723,10 @@
         <v>1</v>
       </c>
       <c r="D14" t="n">
-        <v>711</v>
+        <v>692</v>
       </c>
       <c r="E14" t="n">
-        <v>1.885228199999801</v>
+        <v>1.258504499999617</v>
       </c>
     </row>
     <row r="15">
@@ -744,10 +744,10 @@
         <v>1</v>
       </c>
       <c r="D15" t="n">
-        <v>980</v>
+        <v>964</v>
       </c>
       <c r="E15" t="n">
-        <v>15.25094390000049</v>
+        <v>7.117369999999937</v>
       </c>
     </row>
     <row r="16">
@@ -765,10 +765,10 @@
         <v>1</v>
       </c>
       <c r="D16" t="n">
-        <v>719</v>
+        <v>722</v>
       </c>
       <c r="E16" t="n">
-        <v>40.94512949999989</v>
+        <v>20.66013620000012</v>
       </c>
     </row>
   </sheetData>
@@ -834,17 +834,17 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>7955</v>
+        <v>7871</v>
       </c>
       <c r="D2" t="n">
-        <v>7955</v>
+        <v>7871</v>
       </c>
       <c r="E2" t="n">
-        <v>7955</v>
+        <v>7871</v>
       </c>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="n">
-        <v>0.3334324000006745</v>
+        <v>0.2966114000009838</v>
       </c>
     </row>
     <row r="3">
@@ -859,17 +859,17 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>7662</v>
+        <v>7674</v>
       </c>
       <c r="D3" t="n">
-        <v>7662</v>
+        <v>7674</v>
       </c>
       <c r="E3" t="n">
-        <v>7662</v>
+        <v>7674</v>
       </c>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="n">
-        <v>12.48907169999984</v>
+        <v>8.998690500000521</v>
       </c>
     </row>
     <row r="4">
@@ -884,17 +884,17 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>8495</v>
+        <v>8342</v>
       </c>
       <c r="D4" t="n">
-        <v>8495</v>
+        <v>8342</v>
       </c>
       <c r="E4" t="n">
-        <v>8495</v>
+        <v>8342</v>
       </c>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="n">
-        <v>4.900403800000277</v>
+        <v>5.168920899999648</v>
       </c>
     </row>
     <row r="5">
@@ -909,17 +909,17 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>675</v>
+        <v>686</v>
       </c>
       <c r="D5" t="n">
-        <v>675</v>
+        <v>686</v>
       </c>
       <c r="E5" t="n">
-        <v>675</v>
+        <v>686</v>
       </c>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="n">
-        <v>3.794308999999885</v>
+        <v>4.112357500000144</v>
       </c>
     </row>
     <row r="6">
@@ -934,17 +934,17 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>681</v>
+        <v>689</v>
       </c>
       <c r="D6" t="n">
-        <v>681</v>
+        <v>689</v>
       </c>
       <c r="E6" t="n">
-        <v>681</v>
+        <v>689</v>
       </c>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="n">
-        <v>129.007764</v>
+        <v>65.01397750000069</v>
       </c>
     </row>
     <row r="7">
@@ -959,17 +959,17 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>958</v>
+        <v>1009</v>
       </c>
       <c r="D7" t="n">
-        <v>958</v>
+        <v>1009</v>
       </c>
       <c r="E7" t="n">
-        <v>958</v>
+        <v>1009</v>
       </c>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="n">
-        <v>15.42478030000075</v>
+        <v>12.76222730000154</v>
       </c>
     </row>
     <row r="8">
@@ -984,17 +984,17 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>22483</v>
+        <v>22442</v>
       </c>
       <c r="D8" t="n">
-        <v>22483</v>
+        <v>22442</v>
       </c>
       <c r="E8" t="n">
-        <v>22483</v>
+        <v>22442</v>
       </c>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="n">
-        <v>10.74744179999925</v>
+        <v>4.652482800000143</v>
       </c>
     </row>
     <row r="9">
@@ -1009,17 +1009,17 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>22857</v>
+        <v>22879</v>
       </c>
       <c r="D9" t="n">
-        <v>22857</v>
+        <v>22879</v>
       </c>
       <c r="E9" t="n">
-        <v>22857</v>
+        <v>22879</v>
       </c>
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="n">
-        <v>131.9376242999997</v>
+        <v>62.5200748999996</v>
       </c>
     </row>
     <row r="10">
@@ -1034,17 +1034,17 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>33203</v>
+        <v>33940</v>
       </c>
       <c r="D10" t="n">
-        <v>33203</v>
+        <v>33940</v>
       </c>
       <c r="E10" t="n">
-        <v>33203</v>
+        <v>33940</v>
       </c>
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="n">
-        <v>26.97715880000032</v>
+        <v>12.71414080000068</v>
       </c>
     </row>
     <row r="11">
@@ -1059,17 +1059,17 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>1369</v>
+        <v>1314</v>
       </c>
       <c r="D11" t="n">
-        <v>1369</v>
+        <v>1314</v>
       </c>
       <c r="E11" t="n">
-        <v>1369</v>
+        <v>1314</v>
       </c>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="n">
-        <v>8.247546900000088</v>
+        <v>4.023495299999922</v>
       </c>
     </row>
     <row r="12">
@@ -1084,17 +1084,17 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>1280</v>
+        <v>1292</v>
       </c>
       <c r="D12" t="n">
-        <v>1280</v>
+        <v>1292</v>
       </c>
       <c r="E12" t="n">
-        <v>1280</v>
+        <v>1292</v>
       </c>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="n">
-        <v>119.1917635</v>
+        <v>56.92731110000022</v>
       </c>
     </row>
     <row r="13">
@@ -1109,17 +1109,17 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>1888</v>
+        <v>1853</v>
       </c>
       <c r="D13" t="n">
-        <v>1888</v>
+        <v>1853</v>
       </c>
       <c r="E13" t="n">
-        <v>1888</v>
+        <v>1853</v>
       </c>
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="n">
-        <v>18.93730810000034</v>
+        <v>12.24914619999981</v>
       </c>
     </row>
     <row r="14">
@@ -1134,17 +1134,17 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>711</v>
+        <v>692</v>
       </c>
       <c r="D14" t="n">
-        <v>711</v>
+        <v>692</v>
       </c>
       <c r="E14" t="n">
-        <v>711</v>
+        <v>692</v>
       </c>
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="n">
-        <v>1.885228199999801</v>
+        <v>1.258504499999617</v>
       </c>
     </row>
     <row r="15">
@@ -1159,17 +1159,17 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>719</v>
+        <v>722</v>
       </c>
       <c r="D15" t="n">
-        <v>719</v>
+        <v>722</v>
       </c>
       <c r="E15" t="n">
-        <v>719</v>
+        <v>722</v>
       </c>
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="n">
-        <v>40.94512949999989</v>
+        <v>20.66013620000012</v>
       </c>
     </row>
     <row r="16">
@@ -1184,17 +1184,17 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>980</v>
+        <v>964</v>
       </c>
       <c r="D16" t="n">
-        <v>980</v>
+        <v>964</v>
       </c>
       <c r="E16" t="n">
-        <v>980</v>
+        <v>964</v>
       </c>
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="n">
-        <v>15.25094390000049</v>
+        <v>7.117369999999937</v>
       </c>
     </row>
   </sheetData>

</xml_diff>